<commit_message>
Added mapping between ADs and Capabilities. Staretd mapping BRs to DDs from completed HLD DD doc
</commit_message>
<xml_diff>
--- a/docs/project-management/03_Design/hld/Northwind-Design-Decision-Points-Register.xlsx
+++ b/docs/project-management/03_Design/hld/Northwind-Design-Decision-Points-Register.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/03_Design/hld/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="8_{2C3502F3-4C45-4823-AC68-A5DDF768DFBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{614C1E6E-4E43-4E28-BA4E-1DF11163120A}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="8_{2C3502F3-4C45-4823-AC68-A5DDF768DFBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E169F4BB-D7DD-42DE-98BB-C546AADD2056}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1A4B7B0D-60EB-4FD5-9CB7-F59658F0FC54}"/>
   </bookViews>
   <sheets>
     <sheet name="Design Decision Register" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
-    <sheet name="Glossary" sheetId="2" r:id="rId3"/>
+    <sheet name="Glossary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="133">
   <si>
     <t>Decision ID</t>
   </si>
@@ -416,9 +415,6 @@
     <t>CAP-015 Compute Provisioning / Hosting; CAP-010 Application Hosting; requirements for infrastructure scalability, standardisation, recoverability and supportability; CON-005 Operational Consistency; CON-011 Scalable Without Unnecessary Complexity; CON-012 Supportable &amp; Maintainable Design; DP-002 Prefer Simplicity; DP-003 Standardise Where Practical; DP-013 Design for Managed Growth; v1 focus on Linux/RHCSA administration.</t>
   </si>
   <si>
-    <t>1. KVM + libvirt — direct Linux virtualisation stack managed through Linux tooling/APIs. 2. Proxmox VE — integrated virtualisation management platform built around KVM and related open-source technologies. 3. VMware/ESXi — established enterprise virtualisation platform; retained as a comparison option but not preferred for v1 due to licensing/access considerations and project fit.</t>
-  </si>
-  <si>
     <t>Requirements/capability fit; deployment complexity; administrative overhead; Linux/RHCSA learning alignment; workload isolation; scalability; recoverability; hardware compatibility; management usability; cost/licensing; supportability; ability to expand the lab later.</t>
   </si>
   <si>
@@ -449,12 +445,6 @@
     <t>Identity &amp; Access Management Architecture</t>
   </si>
   <si>
-    <t>CAP-001 Identity &amp; Access Management; CAP-016 Systems Administration &amp; Management; requirements for user lifecycle management, role-based access, secure data access and administrative access; Security, Maintainability and Operational Consistency NFRs; CON-002 Least-Privilege Access; CON-005 Operational Consistency &amp; Standardisation; CON-012 Supportable &amp; Maintainable Design; DP-002 Prefer Simplicity; DP-003 Standardise Where Practical; DP-006 Enforce Least Privilege; DP-009 Treat Administrative Access as a Controlled Service; DP-015 Prefer Automation for Repeatable Operations, Not Understanding Replacement.</t>
-  </si>
-  <si>
-    <t>1. Local Linux IAM — identities, groups, permissions and privileged access maintained independently on each Linux host using native Linux mechanisms. 2. Local Linux IAM with centralised automation — retain local identities while using automation to distribute and maintain standardised account/group/access configuration across systems. 3. Centralised IAM — introduce a shared directory/identity service providing central authentication and identity lifecycle management across supported systems.</t>
-  </si>
-  <si>
     <t>Requirements fit; security and least privilege; RHCSA learning alignment; implementation complexity; administrative overhead; user lifecycle management; consistency across systems; scalability; supportability; recoverability; automation potential; risk of configuration/account drift; suitability for Northwind v1 scale.</t>
   </si>
   <si>
@@ -467,17 +457,1054 @@
     <t>Local identities must be maintained across multiple systems, increasing administrative effort as the environment grows. Account, UID/GID, group and privilege configuration may drift between hosts if standards are not followed. Joiner/mover/leaver processes must ensure accounts are updated or disabled on every applicable system, creating a risk of orphaned accounts. Automation can reduce these risks but does not provide true central authentication and introduces its own operational dependency. Centralised IAM may therefore become preferable as Northwind's infrastructure grows.</t>
   </si>
   <si>
-    <t>Decision Owner / Approver</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">if host/user numbers, joiner-mover-leaver workload, identity drift, security risk, or administrative effort become unacceptable, Northwind should reassess </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
+    <t>File &amp; Data Services Architecture</t>
+  </si>
+  <si>
+    <t>CAP-003 File &amp; Data Services; CAP-001 Identity &amp; Access Management; CAP-004 Storage Provisioning &amp; Management; requirements for secure file services, structured data organisation, departmental data segregation and secure data access; Data Protection, Security, Recoverability and Operational Consistency NFRs; CON-002 Least-Privilege Access; CON-005 Operational Consistency &amp; Standardisation; CON-013 Business Data Segregation &amp; Protection; DP-002 Prefer Simplicity; DP-003 Standardise Where Practical; DP-006 Enforce Least Privilege; DP-012 Avoid Unnecessary Coupling; DP-017 Protect Business Data Throughout its Lifecycle.</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Consolidated Linux file-services node</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — a Linux server provides appropriate file-sharing services directly to supported clients, with native Linux permissions and access-control mechanisms protecting departmental data. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Separated storage and file-services architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — dedicated storage services provide storage to a separate file-services node, which provides client-facing file access and access controls. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Cloud-integrated file services</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — locally hosted file services combined with cloud-based synchronisation/versioning for selected business data.</t>
+    </r>
+  </si>
+  <si>
+    <t>Business requirements fit; Windows/Linux client interoperability; security and departmental segregation; least-privilege enforcement; operational complexity; supportability; recoverability; scalability; failure dependencies; administrative overhead; RHCSA/Linux learning alignment; integration with IAM; integration with backup/recovery; future extensibility.</t>
+  </si>
+  <si>
+    <t>Consolidated Linux file-services architecture using appropriate Linux/Windows-compatible file-sharing protocols and native Linux access controls, backed by managed persistent storage.</t>
+  </si>
+  <si>
+    <t>A consolidated Linux file-services architecture satisfies Northwind's current requirements for shared file access, structured departmental data and controlled access without introducing an unnecessary separate storage-services tier. The architecture supports Linux-native ownership, group permissions, ACLs and host security controls while allowing appropriate file-sharing protocols to support both Linux and Windows clients. It provides strong alignment with the v1 Linux/RHCSA learning objectives while maintaining a comparatively simple and supportable operational model. Storage implementation is intentionally treated as a separate architectural decision.</t>
+  </si>
+  <si>
+    <t>Combining file-service functionality on a single logical service node creates a service dependency and potential single point of failure unless resilience or recovery controls mitigate the risk. Native access controls and client-facing file-sharing configuration must remain aligned to prevent unintended access. As data volumes, performance requirements or availability requirements increase, separation of storage and file-service responsibilities may become justified. Cloud integration is deferred and may require future reassessment if Northwind develops requirements for external collaboration, cloud-based versioning or additional off-site data capabilities.</t>
+  </si>
+  <si>
+    <t>DD-004</t>
+  </si>
+  <si>
+    <t>Storage Architecture</t>
+  </si>
+  <si>
+    <t>CAP-004 Storage Provisioning &amp; Management; CAP-003 File &amp; Data Services; CAP-007 Backup &amp; Recovery; requirements for structured data organisation, departmental data segregation, capacity management, recoverability and infrastructure scalability; Performance, Scalability, Data Protection, Recoverability and Operational Consistency NFRs; CON-003 Recoverable Operations; CON-005 Operational Consistency &amp; Standardisation; CON-011 Scalable Without Unnecessary Complexity; CON-012 Supportable &amp; Maintainable Design; CON-013 Business Data Segregation &amp; Protection; CON-014 Capacity &amp; Performance Visibility; DP-002 Prefer Simplicity; DP-003 Standardise Where Practical; DP-004 Design for Recoverability; DP-013 Design for Managed Growth; DP-016 Design for Supportability; DP-017 Protect Business Data Throughout its Lifecycle.</t>
+  </si>
+  <si>
+    <t>Requirements fit; capacity growth; storage isolation; recoverability; operational complexity; performance; scalability; supportability; filesystem flexibility; quota capability; snapshot/recovery options; failure dependencies; RHCSA/Linux learning alignment; integration with file services; integration with backup/recovery; future extensibility.</t>
+  </si>
+  <si>
+    <t>Locally presented LVM-backed XFS storage for v1, with business data logically separated and separate filesystems introduced only where capacity, recovery, security or operational isolation requirements justify them. A dedicated storage-services node and higher-level storage-management abstraction are deferred.</t>
+  </si>
+  <si>
+    <t>LVM and XFS provide a mature and flexible Linux-native storage architecture that supports Northwind's current capacity, growth, organisation and recoverability requirements without introducing an unnecessary network-storage tier. LVM provides controlled allocation and expansion of storage while XFS provides a robust filesystem suited to the planned Linux environment. The architecture also strongly supports v1 Linux/RHCSA learning objectives by exposing administrators directly to logical volumes, filesystems, mounts, capacity management and storage troubleshooting. Departmental organisation does not itself require a filesystem per department; the final logical-volume and filesystem layout will therefore be determined during LLD based on capacity, recovery and isolation requirements.</t>
+  </si>
+  <si>
+    <t>Locally presented storage creates a dependency on the workload/compute environment and does not provide the separation available from dedicated network storage. Poor initial volume sizing may require later capacity changes. Multiple departmental filesystems would provide stronger storage-level isolation but increase administration and may create inefficient capacity allocation. LVM snapshots can assist some operational recovery scenarios but do not replace independent backups. Deferring a dedicated storage tier limits some future scalability and resilience options but avoids unnecessary v1 complexity.</t>
+  </si>
+  <si>
+    <t>DD-005</t>
+  </si>
+  <si>
+    <t>Backup &amp; Recovery Architecture</t>
+  </si>
+  <si>
+    <t>CAP-007 Backup &amp; Recovery; CAP-003 File &amp; Data Services; CAP-004 Storage Provisioning &amp; Management; CAP-015 Compute Provisioning / Hosting; requirements for business continuity backups, backup validation and recovery testing, service recovery and recoverable operations; Availability, Reliability, Data Protection and Recoverability NFRs; CON-003 Recoverable Operations; CON-004 Proportionate Availability &amp; Resilience; CON-008 Controlled &amp; Recoverable Change; CON-013 Business Data Segregation &amp; Protection; DP-004 Design for Recoverability; DP-005 Apply Proportionate Resilience; DP-010 Prefer Controlled &amp; Reversible Change; DP-017 Protect Business Data Throughout its Lifecycle.</t>
+  </si>
+  <si>
+    <t>Business requirements fit; RPO/RTO capability; protection against accidental deletion, corruption, administrative error, workload loss, storage failure and infrastructure failure; recovery granularity; backup isolation; security; recoverability; restore testing; retention capability; operational complexity; monitoring/reporting; storage requirements; scalability; supportability; Linux/RHCSA learning alignment; integration with compute, storage and file services.</t>
+  </si>
+  <si>
+    <t>Layered backup and recovery architecture comprising short-term point-in-time recovery mechanisms, a dedicated backup service using protected backup storage, and a secondary backup copy maintained outside the primary production failure domain. Backup effectiveness will be validated through scheduled restore testing and documented recovery procedures.</t>
+  </si>
+  <si>
+    <t>A layered architecture provides protection against a broader range of failure scenarios than any single backup mechanism. Short-term point-in-time recovery provides rapid rollback for appropriate operational errors or changes, while an independent backup service and protected repository provide recoverability following data corruption, workload loss or production-storage failure. A secondary copy outside the primary failure domain provides additional protection against loss of the primary compute/storage environment. The approach supports protection at appropriate levels, including business data, system/configuration data and recoverable workload state, while allowing recovery methods and schedules to be aligned with Northwind's RPO/RTO requirements. Scheduled restore testing ensures that backup success is demonstrated through actual recoverability rather than backup-job status alone.</t>
+  </si>
+  <si>
+    <t>The layered architecture introduces additional infrastructure, storage consumption and administrative overhead compared with a simple backup approach. Snapshots or other point-in-time mechanisms remain dependent on their underlying storage and must not be treated as independent backups. A remote secondary copy does not automatically provide protection against malicious deletion or ransomware unless appropriate isolation, credentials and access controls are implemented. Backup capacity will increase according to protected data volume, backup frequency and retention requirements. Recovery procedures must be maintained and tested. Service-specific RPO/RTO values remain to be refined and may affect the eventual backup schedules, retention and recovery mechanisms selected during LLD.</t>
+  </si>
+  <si>
+    <t>DD-006</t>
+  </si>
+  <si>
+    <t>Monitoring &amp; Alerting Architecture</t>
+  </si>
+  <si>
+    <t>CAP-006 Infrastructure Monitoring &amp; Alerting; CAP-012 Reporting; CAP-015 Compute Provisioning / Hosting; CAP-016 Systems Administration &amp; Management; requirements for operational monitoring and alerting, capacity and performance management, reporting and visibility, service recovery and incident investigation/troubleshooting; Availability, Reliability, Performance, Supportability and Monitoring &amp; Observability NFRs; CON-006 Observable &amp; Auditable Operations; CON-012 Supportable &amp; Maintainable Design; CON-014 Capacity &amp; Performance Visibility; DP-008 Make Operations Observable &amp; Auditable; DP-013 Design for Managed Growth; DP-016 Design for Supportability.</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Native/decentralised Linux monitoring</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — administrators use native Linux tools, scripts and scheduled checks to assess individual host and service health. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Dedicated central monitoring platform</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — infrastructure and service telemetry is collected centrally to provide continuous visibility, alerting, historical data and reporting. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Hybrid monitoring architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — centralised monitoring provides continuous visibility, alerting, historical trends and capacity reporting, while native Linux tools remain available for detailed host-level diagnosis and troubleshooting.</t>
+    </r>
+  </si>
+  <si>
+    <t>Requirements fit; infrastructure and service visibility; proactive fault detection; service-health monitoring; alerting and escalation capability; historical metric retention; capacity/performance trending; reporting capability; Linux/RHCSA learning alignment; troubleshooting capability; operational complexity; security; scalability; supportability; monitoring-platform dependencies; integration with backup, compute, storage, networking and future application services.</t>
+  </si>
+  <si>
+    <t>Hybrid monitoring architecture consisting of a centralised monitoring and alerting service providing infrastructure and service health visibility, historical capacity/performance data, configurable threshold-based alerting and operational reporting across supported systems. Native Linux diagnostic and troubleshooting tools will remain the primary mechanism for detailed host-level investigation.</t>
+  </si>
+  <si>
+    <t>A hybrid approach provides Northwind with central operational visibility while preserving direct Linux administration and troubleshooting capability. Central monitoring enables proactive detection of host, service, storage, backup, network and resource issues; maintains historical data for capacity and performance analysis; and allows alerts to be routed to IT when defined warning or critical conditions occur. Native Linux tools complement this capability by enabling administrators to investigate the underlying cause of detected conditions directly on affected systems. This approach satisfies Northwind's monitoring, reporting and capacity-management requirements without making the monitoring platform a replacement for administrator understanding of the underlying Linux systems.</t>
+  </si>
+  <si>
+    <t>A central monitoring service introduces an additional infrastructure component that must itself be secured, patched, backed up and maintained. Failure of the monitoring platform may reduce operational visibility and create a monitoring blind spot; appropriate health checks or independent operational controls should therefore be considered. Excessive or poorly configured thresholds may cause alert fatigue, while insufficient thresholds may allow significant conditions to go undetected. Collection and retention of detailed historical metrics will consume storage and compute resources. Agent versus agentless collection, metric retention periods, thresholds, alert-routing mechanisms and monitoring-platform technology remain to be determined during subsequent design activities.</t>
+  </si>
+  <si>
+    <t>DD-007</t>
+  </si>
+  <si>
+    <t>Logging &amp; Audit Architecture</t>
+  </si>
+  <si>
+    <t>CAP-005 Logging &amp; Audit; CAP-006 Infrastructure Monitoring &amp; Alerting; CAP-014 Time Synchronisation Services; CAP-016 Systems Administration &amp; Management; CAP-017 Security; requirements for centralised logging, incident investigation/troubleshooting, reporting and visibility, secure administration and threat detection; Security, Auditability, Supportability, Monitoring &amp; Observability and Time Consistency NFRs; CON-006 Observable &amp; Auditable Operations; CON-007 Consistent Time Reference; CON-012 Supportable &amp; Maintainable Design; CON-013 Business Data Segregation &amp; Protection; DP-008 Make Operations Observable &amp; Auditable; DP-016 Design for Supportability; DP-018 Time Is a Shared Infrastructure Dependency.</t>
+  </si>
+  <si>
+    <t>Requirements fit; operational troubleshooting capability; security/audit traceability; cross-system investigation; retention capability; log integrity and protection; availability during central-service failure; time consistency; secure transport; access control; storage/capacity requirements; privacy and data protection; monitoring integration; operational complexity; supportability; scalability; Linux/RHCSA learning alignment; future extensibility toward more advanced analytics or threat detection.</t>
+  </si>
+  <si>
+    <t>Hybrid logging and audit architecture in which supported Linux systems maintain native local system, service and security audit records while selected operational and security events are securely forwarded to a central logging service. The central service will provide protected longer-term retention and cross-system investigation capability, supported by consistent infrastructure time, appropriate access controls and defined audit policy. Selected significant events may integrate with monitoring and alerting where timely operational response is required.</t>
+  </si>
+  <si>
+    <t>The hybrid approach preserves native Linux logging and auditing capabilities for immediate host-level troubleshooting while providing Northwind with centralised retention and investigation of important events across multiple systems. Central forwarding reduces dependence on the originating host remaining available and improves the ability to reconstruct incidents spanning multiple services. Consistent time synchronisation allows events from different systems to be correlated reliably. Native Linux logging and auditing also provide strong alignment with v1 Linux/RHCSA learning objectives while avoiding the additional complexity of introducing a full-scale log analytics or SIEM platform before such capability is justified. Integration with monitoring allows selected operational or security events requiring immediate action to generate alerts without conflating the monitoring and logging capabilities.</t>
+  </si>
+  <si>
+    <t>A central logging service introduces an additional infrastructure component that must itself be secured, monitored, patched, backed up and capacity-managed. Centralisation creates a repository containing potentially sensitive operational and security information and therefore requires restricted administrative access and appropriate data protection. Loss of the central logging service may temporarily reduce cross-system visibility; local retention/buffering should therefore preserve records where practical until forwarding can resume. Excessive logging or audit rules may generate unnecessary storage consumption and operational noise, while insufficient logging may leave gaps during</t>
+  </si>
+  <si>
+    <t>DD-008</t>
+  </si>
+  <si>
+    <t>Remote &amp; Administrative Access Architecture</t>
+  </si>
+  <si>
+    <t>CAP-008 Remote Access; CAP-001 Identity &amp; Access Management; CAP-009 Network Connectivity &amp; Core Network Services; CAP-016 Systems Administration &amp; Management; CAP-017 Security; requirements for secure remote access, remote administration, network security, administrative approval/control, consistent remote-user access and incident investigation; Security, Auditability, Supportability, Recoverability and Operational Consistency NFRs; CON-002 Least-Privilege Access; CON-006 Observable &amp; Auditable Operations; CON-009 Secure Administrative Access; CON-012 Supportable &amp; Maintainable Design; DP-006 Enforce Least Privilege; DP-007 Use Defence in Depth; DP-009 Treat Administrative Access as a Controlled Service; DP-016 Design for Supportability.</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Direct remote access to individual services and SSH endpoints</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — users and administrators connect directly to exposed services as required. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Common secure remote-access service with limited distinction between user and administrator paths</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — all remote users enter through the same access mechanism with subsequent access controlled internally. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Secure remote-access architecture with a distinct trusted administrative path</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — ordinary users access permitted business services through office or remote-access networks, while Linux administration is restricted to trusted administrative networks or equivalent controlled remote-access policies and uses named administrative identities with controlled privilege elevation. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4. Dedicated jump/bastion architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — administrative access must traverse a dedicated management host before reaching target systems.</t>
+    </r>
+  </si>
+  <si>
+    <t>Security; attack-surface reduction; least privilege; separation of user and administrative access; administrative traceability; remote-user usability; support for office and remote working; identity/accountability; privilege control; network and host-level enforcement; logging/audit integration; recovery access; operational complexity; resilience; supportability; scalability; Linux/RHCSA learning alignment; future extensibility toward MFA, bastion hosts or stronger management-plane isolation.</t>
+  </si>
+  <si>
+    <t>Northwind will provide secure remote access for users and administrators through a controlled remote-access service. Ordinary users will be restricted to authorised business services, while privileged Linux administration will be limited to trusted administrative networks or equivalent controlled remote-access paths. Administrative access will use named identities, strong authentication and controlled privilege elevation rather than direct root login. Network-level and host-level security controls will restrict permitted administrative sources, and remote-access, SSH and privileged administrative activity will be integrated with central logging and audit. A controlled recovery-access mechanism will be maintained for situations where normal administrative access is unavailable.</t>
+  </si>
+  <si>
+    <t>The proposed architecture provides secure remote working while maintaining a stronger control boundary around privileged administration. Separating ordinary user access from administrative access reduces the likelihood that compromised user devices or accounts can directly reach management services. Named administrative identities and controlled privilege elevation improve accountability and support least-privilege operation, while network and host-level controls provide defence in depth. Integration with logging and audit supports investigation and traceability. The approach remains proportionate for Northwind v1 by avoiding the additional infrastructure and dependencies associated with a dedicated bastion or privileged-access platform, while preserving a clear migration path should stronger controls later become necessary. It also provides strong alignment with Linux/RHCSA learning through SSH administration, user/group management, sudo, host firewalls and troubleshooting.</t>
+  </si>
+  <si>
+    <t>The remote-access service becomes an important dependency for remote users and administrators and must itself be secured, monitored and maintained. Incorrect firewall or access policy could either expose administrative services too broadly or prevent legitimate administration. SSH key or credential lifecycle must be managed carefully. Under DD-002, local Linux identities mean administrative accounts remain distributed across hosts unless later automation or central IAM is introduced. A recovery-access mechanism is necessary but must not become an uncontrolled bypass of normal security controls. The absence of a dedicated jump host reduces architectural complexity but provides fewer central control points than a more mature privileged-access design. Exact network ranges, VPN policies, firewall rules, SSH settings, authentication mechanisms and recovery procedures will be defined during LLD.</t>
+  </si>
+  <si>
+    <t>DD-009</t>
+  </si>
+  <si>
+    <t>Network Security &amp; Segmentation Architecture</t>
+  </si>
+  <si>
+    <t>CAP-009 Network Connectivity &amp; Core Network Services; CAP-008 Remote Access; CAP-016 Systems Administration &amp; Management; CAP-017 Security; requirements for Network Security, Network Segmentation, Secure Remote Access, Secure Remote Administration, Network Resource Access and Host Security Enforcement; Security, Data Protection, Availability, Supportability and Operational Consistency NFRs; CON-001 Security by Design; CON-002 Least-Privilege Access; CON-006 Observable &amp; Auditable Operations; CON-009 Secure Administrative Access; CON-011 Scalable Without Unnecessary Complexity; CON-013 Business Data Segregation &amp; Protection; DP-002 Prefer Simplicity Over Unnecessary Complexity; DP-006 Enforce Least Privilege; DP-007 Use Defence in Depth; DP-009 Treat Administrative Access as a Controlled Service; DP-012 Avoid Unnecessary Coupling; DP-013 Design for Managed Growth.</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Flat / minimally segmented network</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — users, servers and management services operate within a largely common trust environment with limited traffic separation. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Functionally segmented network with controlled inter-zone access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — systems are separated into meaningful trust/function zones, with default-deny inter-zone policy and explicitly authorised service flows. Network controls are supplemented by host-level security. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Highly segmented / microsegmented architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — workloads and potentially individual systems/endpoints receive fine-grained isolation and policy enforcement, substantially reducing lateral movement but increasing design and operational complexity.</t>
+    </r>
+  </si>
+  <si>
+    <t>Security; least privilege; reduction of attack surface and lateral-movement opportunities; protection of administrative interfaces; business/service connectivity requirements; remote-access integration; defence in depth; operational simplicity; troubleshooting complexity; scalability; supportability; availability; logging and monitoring capability; Linux/RHCSA learning alignment; compatibility with existing network requirements; ability to introduce additional zones or stronger segmentation as Northwind grows.</t>
+  </si>
+  <si>
+    <t>Northwind will adopt a functionally segmented network architecture using distinct User, Server/Infrastructure, Management/Administrative and External/Untrusted trust zones. Inter-zone communication will follow a least-privilege, default-deny model, with only explicitly required service flows permitted. Network-level policy enforcement will be supplemented by Linux host firewall controls and SELinux-based host security to provide defence in depth. Infrastructure management interfaces and administrative services will only be accessible through trusted administrative paths. Remote users and administrators will enter equivalent user or administrative trust contexts through the secure remote-access architecture defined by DD-008. Unsolicited inbound Internet access will not be permitted in v1, and significant network/security events will be integrated with central logging and monitoring.</t>
+  </si>
+  <si>
+    <t>Functional segmentation provides materially stronger isolation than a flat network while remaining proportionate to Northwind's current size and operational capability. Separating ordinary users, internal services and privileged management reduces the potential blast radius of compromised endpoints or accounts and prevents user networks from unnecessarily reaching administrative interfaces. A default-deny inter-zone model ensures connectivity is provided according to defined service requirements rather than broad network trust. Combining network policy with Linux host firewall controls provides defence in depth, while SELinux provides an additional process/resource security boundary if a host service is compromised. The model integrates naturally with DD-008 by preserving user and administrative trust boundaries for remote access and supports DD-006/DD-007 through monitoring and logging of significant network events. The design avoids the operational complexity of full microsegmentation while retaining a clear path to additional segmentation as Northwind grows.</t>
+  </si>
+  <si>
+    <t>Segmentation increases firewall-policy, documentation and troubleshooting requirements compared with a flat network. Incorrect policy may either expose services unnecessarily or disrupt legitimate dependencies. Default-deny operation requires service flows to be identified and maintained as the environment changes. Functional zones reduce cross-zone lateral movement but do not inherently prevent communication between systems within the same zone; endpoint/workload-level microsegmentation is therefore outside v1. The Management/Admin zone represents a high-trust environment and requires particularly strong access controls. Additional zones may become necessary as applications, infrastructure or externally accessible services grow. Exact VLANs, subnets, routing, firewall rules, permitted source/destination/port matrices, VPN address pools and Linux host-firewall configuration will be defined during LLD.</t>
+  </si>
+  <si>
+    <t>DD-010</t>
+  </si>
+  <si>
+    <t>Patch &amp; Software Lifecycle Management Architecture</t>
+  </si>
+  <si>
+    <t>CAP-013 Software &amp; Patch Management; CAP-016 Systems Administration &amp; Management; CAP-018 Asset &amp; Configuration Management; CAP-007 Backup &amp; Recovery; CAP-012 Reporting; requirements for Software and System Update Management, Software and Package Lifecycle Management, Administrative Approval Workflows, Operational Documentation and Incident Investigation/Troubleshooting; Security, Maintainability, Recoverability, Supportability, Operational Consistency and Auditability NFRs; CON-003 Recoverable Operations; CON-005 Operational Consistency &amp; Standardisation; CON-008 Controlled &amp; Recoverable Change; CON-012 Supportable &amp; Maintainable Design; DP-003 Standardise Where Practical; DP-004 Design for Recoverability; DP-010 Prefer Controlled &amp; Reversible Change; DP-015 Prefer Automation for Repeatable Operations, Not Understanding Replacement; DP-016 Design for Supportability.</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Decentralised/manual host patching</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — administrators patch each Linux system independently using native package-management tools and approved repositories. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Controlled native Linux lifecycle process</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — approved software sources, role-based package baselines, documented patch cadence, sandbox-first validation, approval, controlled production deployment, verification, reporting and defined recovery procedures using native Linux administration tooling. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Centralised enterprise lifecycle-management platform</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — dedicated infrastructure centrally manages repositories, patch staging, deployment, compliance, inventory and reporting across systems.</t>
+    </r>
+  </si>
+  <si>
+    <t>Security; trusted software provenance; consistency; operational control; change governance; testing capability; recovery readiness; service availability; reboot impact; post-change validation; reporting and traceability; exception management; supportability; scalability; operational complexity; RHCSA/Linux learning alignment; automation potential; compatibility with the v1 environment.</t>
+  </si>
+  <si>
+    <t>Northwind will adopt a controlled native Linux software and patch lifecycle using approved and trusted software sources, role-based software baselines and documented change processes. Routine updates will follow a defined monthly maintenance cycle incorporating assessment, sandbox-first validation, approval, controlled production deployment, post-change verification and reporting. Critical security updates may follow an accelerated change path while retaining appropriate testing, approval and recovery controls. Production changes will have defined recovery procedures aligned with the Backup &amp; Recovery architecture, including consideration of reboot and service-availability requirements. Software-source and package deviations will be controlled and documented. Initial operations will use native Linux package-management and diagnostic capabilities through manual, repeatable procedures, with automation introduced where operational scale and maturity justify it.</t>
+  </si>
+  <si>
+    <t>The controlled native Linux lifecycle model provides Northwind with significantly stronger governance and consistency than ad-hoc host patching while avoiding the complexity of introducing a dedicated enterprise lifecycle-management platform in v1. Restricting systems to approved software sources improves security and supportability, while role-based package baselines reduce configuration drift and unnecessary software variation. Sandbox-first validation reduces the risk of production disruption, and differentiated routine versus urgent-security paths allow Northwind to balance operational stability with timely remediation of critical vulnerabilities. Defined recovery and post-change validation ensure patch success is measured by restoration of the business service rather than package installation alone. The model also strongly supports v1 RHCSA objectives by retaining direct administration of packages, repositories, services, logs and recovery procedures before higher levels of automation are introduced.</t>
+  </si>
+  <si>
+    <t>Manual and repeatable native processes require more administrative effort than a central lifecycle-management platform and become harder to scale as the number of hosts increases. Inconsistent execution could create configuration drift unless baselines, procedures and reporting are maintained. Monthly patch cycles may be too slow for critical vulnerabilities, requiring an accelerated security-update process. Package or application dependencies may prevent some patches from being applied immediately; such cases require documented exceptions, risk ownership and periodic review. Kernel or other updates may require reboot and planned service interruption. Recovery methods vary by workload and may involve package remediation, configuration restoration, service-specific recovery, system restoration or rebuild; therefore recovery procedures must be determined before production deployment. Exact repository definitions, package baselines, maintenance windows, severity thresholds, commands, scripts, reporting formats and exception procedures will be defined during LLD and operational documentation.</t>
+  </si>
+  <si>
+    <t>DD-011</t>
+  </si>
+  <si>
+    <t>Automation &amp; Scheduled Operations Architecture</t>
+  </si>
+  <si>
+    <t>CAP-002 Automation &amp; Scheduled Operations; CAP-016 Systems Administration &amp; Management; CAP-006 Infrastructure Monitoring &amp; Alerting; CAP-005 Logging &amp; Audit; CAP-007 Backup &amp; Recovery; CAP-013 Software &amp; Patch Management; requirements for Administrative Automation, Scheduled Administrative Activities, User Provisioning Automation, Backup &amp; Recovery, Capacity &amp; Performance Management, Software/System Update Management and Operational Documentation; Maintainability, Supportability, Operational Consistency, Recoverable Operations and Auditability NFRs; CON-003 Recoverable Operations; CON-005 Operational Consistency &amp; Standardisation; CON-006 Observable &amp; Auditable Operations; CON-008 Controlled &amp; Recoverable Change; CON-012 Supportable &amp; Maintainable Design; DP-003 Standardise Where Practical; DP-010 Prefer Controlled &amp; Reversible Change; DP-015 Prefer Automation for Repeatable Operations, Not Understanding Replacement; DP-016 Design for Supportability.</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Primarily manual operations</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — administrators execute recurring activities manually according to documented procedures. Provides transparency and simplicity but creates increasing administrative effort and potential inconsistency. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Native Linux automation &amp; scheduling</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — sufficiently understood, repetitive and predictable activities are progressively converted into reusable scripts and executed manually or through native Linux scheduling mechanisms as appropriate. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Centralised configuration-management/orchestration platform</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — multi-host configuration and administrative activities are managed through a dedicated automation framework providing greater centralisation, desired-state management and scalability.</t>
+    </r>
+  </si>
+  <si>
+    <t>Operational consistency; repeatability; administrative efficiency; task predictability; failure impact; recoverability; safe repeat execution/idempotency; observability; logging and alerting; least privilege; credential/secret protection; change governance; sandbox testing; source/version control; documentation; ownership; scheduling and dependency management; troubleshooting complexity; scalability; configuration-drift reduction; RHCSA/Linux learning alignment; future extensibility toward configuration-management and orchestration platforms.</t>
+  </si>
+  <si>
+    <t>Northwind will adopt a native Linux automation and scheduling architecture in which repetitive, predictable and sufficiently understood administrative activities are progressively implemented using reusable scripts and native scheduling mechanisms. Automation will be documented, version-controlled, sandbox-tested and deployed through controlled change processes. Automated activities will operate using least privilege, avoid embedded credentials, support safe repeat execution where practicable, and produce sufficient logging and monitoring to ensure failures are detectable and actionable. High-risk, judgement-based or insufficiently mature processes will remain manually controlled until automation can be safely justified. Scheduled operations will be coordinated to avoid conflicting activities. Centralised configuration-management and orchestration platforms will be deferred until environmental scale, configuration drift or operational workload provides a clear requirement.</t>
+  </si>
+  <si>
+    <t>Native Linux automation provides an appropriate balance between operational consistency, efficiency, simplicity and the project's v1 Linux/RHCSA objectives. Administrators will first understand and document operational procedures before progressively automating repetitive activities, reducing the risk of automating poorly understood processes. Initial candidates include backup execution and verification, health/capacity checks, log housekeeping, update discovery and operational reporting. Native scripting and scheduling retain visibility into Linux behaviour while developing practical skills in shell scripting, services, scheduling, permissions, logging and troubleshooting. Version control, sandbox validation and controlled deployment ensure automation is treated as a managed infrastructure asset rather than unmanaged administrative scripts. Integration with central logging and monitoring ensures automated operations do not fail silently. The architecture provides a deliberate progression toward configuration-management/orchestration platforms when environmental scale and operational requirements justify the additional abstraction and complexity.</t>
+  </si>
+  <si>
+    <t>Native scripts and distributed scheduling require greater administrative effort and provide less centralised control than a configuration-management/orchestration platform. Poorly designed automation can reproduce errors consistently or increase the impact of mistakes; therefore testing, review, least privilege and controlled deployment are required. Automation requiring elevated privileges may increase security exposure and must use only the minimum privileges necessary. Scheduled jobs may conflict with backups, maintenance, patching or other operations unless schedules are coordinated. Scripts may become difficult to support if documentation, ownership and version control are neglected. Not every operation can be made fully idempotent, but safe re-execution should be pursued where practical. Manual handling of higher-risk operations increases administrative workload but preserves human judgement during v1. Centralised configuration management should be reconsidered if host growth, configuration drift, repetitive multi-host administration or operational workload makes the native approach inefficient or unreliable. Exact scripts, execution accounts, schedules, systemd timers/cron configuration, log locations, alert thresholds and operational procedures will be defined during LLD and SOP development.</t>
+  </si>
+  <si>
+    <t>DD-012</t>
+  </si>
+  <si>
+    <t>Availability &amp; Resilience Strategy</t>
+  </si>
+  <si>
+    <t>CAP-007 Backup &amp; Recovery; CAP-006 Infrastructure Monitoring &amp; Alerting; CAP-015 Compute Provisioning / Hosting; CAP-009 Network Connectivity &amp; Core Network Services; CAP-016 Systems Administration &amp; Management; requirements for Business Service Continuity, Business Continuity Backups, Backup Validation &amp; Recovery Testing, Service Recovery, Application Resilience and Infrastructure Scalability; Availability, Reliability, Recoverability, Supportability, Data Protection and Operational Consistency NFRs; CON-003 Recoverable Operations; CON-004 Proportionate Availability &amp; Resilience; CON-011 Scalable Without Unnecessary Complexity; CON-012 Supportable &amp; Maintainable Design; DP-002 Prefer Simplicity Over Unnecessary Complexity; DP-004 Design for Recoverability; DP-005 Apply Proportionate Resilience; DP-012 Avoid Unnecessary Coupling; DP-013 Design for Managed Growth; DP-016 Design for Supportability.</t>
+  </si>
+  <si>
+    <t>Business-service criticality; acceptable downtime; RTO; RPO; data-loss tolerance; planned and unplanned downtime; failure-domain analysis; single points of failure; failure-detection time; recovery time; backup/recovery capability; service and infrastructure dependencies; compute-host failure; data resilience; maintenance requirements; recovery testing; operational complexity; supportability; administrative capability; infrastructure/resource cost; scalability; troubleshooting complexity; RHCSA/Linux learning alignment; ability to introduce additional resilience later without unnecessary redesign.</t>
+  </si>
+  <si>
+    <t>Northwind v1 will adopt a recovery-based resilience architecture as the baseline for infrastructure and business services. Single service instances and a single compute platform will be accepted where service requirements can be satisfied through rapid failure detection, documented recovery, standardised rebuild procedures and the protected backup architecture defined by DD-005. Service criticality and service-specific RTO/RPO requirements will be used to determine whether recovery-based resilience is sufficient; selective redundancy will be introduced only where those requirements cannot reasonably be achieved through recovery alone. Broad high-availability, clustering and replicated infrastructure will be deferred until justified by measured business availability requirements. Recovery procedures will be periodically tested and measured against agreed recovery objectives.</t>
+  </si>
+  <si>
+    <t>A recovery-based model provides a proportionate balance between business continuity, cost, complexity, supportability and the objectives of the v1 environment. Monitoring and alerting defined by DD-006 provide rapid failure detection, while DD-005 provides protected backup and recovery capability. Standardised configurations, documented build procedures and operational runbooks support predictable restoration and rebuild of failed services. This approach avoids introducing clustering, replicated infrastructure or other HA technologies before a demonstrated business requirement exists. It also avoids “fake HA”, where redundant service instances remain dependent on a common single point of failure. Resilience will therefore be determined from end-to-end service dependencies and failure domains rather than simply the number of deployed servers. Where a service-specific RTO/RPO cannot be achieved through recovery, targeted redundancy can subsequently be introduced. This preserves a clear growth path toward redundant compute, services, network infrastructure or other HA mechanisms when justified.</t>
+  </si>
+  <si>
+    <t>The v1 architecture deliberately retains single points of failure. In particular, failure of the single compute host may make multiple hosted services simultaneously unavailable until suitable compute capacity is repaired, replaced or made available and workloads are recovered. Single-instance services such as file services, monitoring, logging, remote access and potentially core network services may remain unavailable during recovery. Backups reduce data-loss and recovery risk but do not provide service availability or automatic failover. Actual recovery times depend on failure detection, diagnosis, replacement capacity, backup availability, administrator capability and successful recovery procedures. Critical infrastructure dependencies such as DNS or network/security services may have wider service impact than their individual workload suggests and must therefore be considered during service-criticality analysis. Recovery procedures that are not regularly tested may fail to achieve expected recovery times. Service-specific RTO/RPO requirements remain to be refined before LLD finalisation; where those objectives cannot be achieved using the recovery-based model, additional resilience must be evaluated. Exact recovery procedures, service classifications, recovery sequencing, failover mechanisms and any future redundant components will be defined during LLD and operational documentation.</t>
+  </si>
+  <si>
+    <t>FC-037 / HLD Action — Service Criticality &amp; RTO/RPO Refinement: Northwind and Redstone must classify supported business/infrastructure services and agree appropriate service-specific recovery objectives before LLD finalisation. The proposed recovery architecture must then be validated against those objectives. Where an objective cannot reasonably be achieved through recovery, selective redundancy must be evaluated.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Locally presented LVM-backed XFS storage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — managed block storage is presented directly to the workload, with LVM providing flexible logical storage management and XFS providing the filesystem layer. 2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Higher-level Linux storage management</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — use a storage-management abstraction such as Stratis to simplify provisioning and lifecycle operations. 3.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Dedicated storage-services architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — separate storage and file-service responsibilities, with a storage node providing storage over the network to client workload nodes. 4. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cloud-integrated storage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — supplement local storage with synchronised or cloud-hosted storage services for selected data.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">KVM + libvirt </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">— direct Linux virtualisation stack managed through Linux tooling/APIs. 2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Proxmox VE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — integrated virtualisation management platform built around KVM and related open-source technologies. 3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">VMware/ESXi </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>— established enterprise virtualisation platform; retained as a comparison option but not preferred for v1 due to licensing/access considerations and project fit.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Local Linux IAM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — identities, groups, permissions and privileged access maintained independently on each Linux host using native Linux mechanisms. 2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Local Linux IAM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>with centralised automation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — retain local identities while using automation to distribute and maintain standardised account/group/access configuration across systems. 3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Centralised IAM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — introduce a shared directory/identity service providing central authentication and identity lifecycle management across supported systems.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Native/simple Linux backup architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — scheduled file and configuration backups using Linux-native mechanisms and protected storage. 2.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Dedicated backup service</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — central backup service/repository providing managed protection, retention and recovery of supported workloads. 3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Layered backup &amp; recovery architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — short-term point-in-time recovery mechanisms combined with a dedicated backup service using protected backup storage and a secondary copy outside the primary production failure domain.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Local Linux logging only</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — system, service and audit records remain on individual hosts and are investigated locally when required. 2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fully centralised logging platform</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — supported systems forward records to a dedicated central platform providing storage, search, analysis and potentially advanced correlation. 3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hybrid Linux logging &amp; audit architecture</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — native Linux system/service logging and security auditing remain available locally while selected operational and security records are securely forwarded to a central logging service for protected retention and cross-system investigation.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Recovery-based resilience</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — services primarily operate as single instances, with resilience provided through monitoring, documented recovery, standardised rebuild procedures and protected backups. 2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Selective redundancy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — recovery remains the baseline, but individual business-critical services or infrastructure dependencies receive additional redundancy where their RTO/RPO cannot reasonably be satisfied through recovery alone. 3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Broad High Availability </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>— redundant compute, services, network dependencies and replicated/shared data infrastructure are implemented to provide automatic or rapid failover across much of the environment.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">if host/user numbers, joiner-mover-leaver workload, identity drift, security risk, or administrative effort become unacceptable, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Northwind should reassess </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -487,7 +1514,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -496,212 +1523,14 @@
     </r>
   </si>
   <si>
-    <t>File &amp; Data Services Architecture</t>
-  </si>
-  <si>
-    <t>CAP-003 File &amp; Data Services; CAP-001 Identity &amp; Access Management; CAP-004 Storage Provisioning &amp; Management; requirements for secure file services, structured data organisation, departmental data segregation and secure data access; Data Protection, Security, Recoverability and Operational Consistency NFRs; CON-002 Least-Privilege Access; CON-005 Operational Consistency &amp; Standardisation; CON-013 Business Data Segregation &amp; Protection; DP-002 Prefer Simplicity; DP-003 Standardise Where Practical; DP-006 Enforce Least Privilege; DP-012 Avoid Unnecessary Coupling; DP-017 Protect Business Data Throughout its Lifecycle.</t>
-  </si>
-  <si>
-    <r>
-      <t>1. Consolidated Linux file-services node</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> — a Linux server provides appropriate file-sharing services directly to supported clients, with native Linux permissions and access-control mechanisms protecting departmental data. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2. Separated storage and file-services architecture</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> — dedicated storage services provide storage to a separate file-services node, which provides client-facing file access and access controls. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3. Cloud-integrated file services</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> — locally hosted file services combined with cloud-based synchronisation/versioning for selected business data.</t>
-    </r>
-  </si>
-  <si>
-    <t>Business requirements fit; Windows/Linux client interoperability; security and departmental segregation; least-privilege enforcement; operational complexity; supportability; recoverability; scalability; failure dependencies; administrative overhead; RHCSA/Linux learning alignment; integration with IAM; integration with backup/recovery; future extensibility.</t>
-  </si>
-  <si>
-    <t>Consolidated Linux file-services architecture using appropriate Linux/Windows-compatible file-sharing protocols and native Linux access controls, backed by managed persistent storage.</t>
-  </si>
-  <si>
-    <t>A consolidated Linux file-services architecture satisfies Northwind's current requirements for shared file access, structured departmental data and controlled access without introducing an unnecessary separate storage-services tier. The architecture supports Linux-native ownership, group permissions, ACLs and host security controls while allowing appropriate file-sharing protocols to support both Linux and Windows clients. It provides strong alignment with the v1 Linux/RHCSA learning objectives while maintaining a comparatively simple and supportable operational model. Storage implementation is intentionally treated as a separate architectural decision.</t>
-  </si>
-  <si>
-    <t>Combining file-service functionality on a single logical service node creates a service dependency and potential single point of failure unless resilience or recovery controls mitigate the risk. Native access controls and client-facing file-sharing configuration must remain aligned to prevent unintended access. As data volumes, performance requirements or availability requirements increase, separation of storage and file-service responsibilities may become justified. Cloud integration is deferred and may require future reassessment if Northwind develops requirements for external collaboration, cloud-based versioning or additional off-site data capabilities.</t>
-  </si>
-  <si>
-    <t>DD-004</t>
-  </si>
-  <si>
-    <t>Storage Architecture</t>
-  </si>
-  <si>
-    <t>CAP-004 Storage Provisioning &amp; Management; CAP-003 File &amp; Data Services; CAP-007 Backup &amp; Recovery; requirements for structured data organisation, departmental data segregation, capacity management, recoverability and infrastructure scalability; Performance, Scalability, Data Protection, Recoverability and Operational Consistency NFRs; CON-003 Recoverable Operations; CON-005 Operational Consistency &amp; Standardisation; CON-011 Scalable Without Unnecessary Complexity; CON-012 Supportable &amp; Maintainable Design; CON-013 Business Data Segregation &amp; Protection; CON-014 Capacity &amp; Performance Visibility; DP-002 Prefer Simplicity; DP-003 Standardise Where Practical; DP-004 Design for Recoverability; DP-013 Design for Managed Growth; DP-016 Design for Supportability; DP-017 Protect Business Data Throughout its Lifecycle.</t>
-  </si>
-  <si>
-    <t>1. Locally presented LVM-backed XFS storage — managed block storage is presented directly to the workload, with LVM providing flexible logical storage management and XFS providing the filesystem layer. 2. Higher-level Linux storage management — use a storage-management abstraction such as Stratis to simplify provisioning and lifecycle operations. 3. Dedicated storage-services architecture — separate storage and file-service responsibilities, with a storage node providing storage over the network to client workload nodes. 4. Cloud-integrated storage — supplement local storage with synchronised or cloud-hosted storage services for selected data.</t>
-  </si>
-  <si>
-    <t>Requirements fit; capacity growth; storage isolation; recoverability; operational complexity; performance; scalability; supportability; filesystem flexibility; quota capability; snapshot/recovery options; failure dependencies; RHCSA/Linux learning alignment; integration with file services; integration with backup/recovery; future extensibility.</t>
-  </si>
-  <si>
-    <t>Locally presented LVM-backed XFS storage for v1, with business data logically separated and separate filesystems introduced only where capacity, recovery, security or operational isolation requirements justify them. A dedicated storage-services node and higher-level storage-management abstraction are deferred.</t>
-  </si>
-  <si>
-    <t>LVM and XFS provide a mature and flexible Linux-native storage architecture that supports Northwind's current capacity, growth, organisation and recoverability requirements without introducing an unnecessary network-storage tier. LVM provides controlled allocation and expansion of storage while XFS provides a robust filesystem suited to the planned Linux environment. The architecture also strongly supports v1 Linux/RHCSA learning objectives by exposing administrators directly to logical volumes, filesystems, mounts, capacity management and storage troubleshooting. Departmental organisation does not itself require a filesystem per department; the final logical-volume and filesystem layout will therefore be determined during LLD based on capacity, recovery and isolation requirements.</t>
-  </si>
-  <si>
-    <t>Locally presented storage creates a dependency on the workload/compute environment and does not provide the separation available from dedicated network storage. Poor initial volume sizing may require later capacity changes. Multiple departmental filesystems would provide stronger storage-level isolation but increase administration and may create inefficient capacity allocation. LVM snapshots can assist some operational recovery scenarios but do not replace independent backups. Deferring a dedicated storage tier limits some future scalability and resilience options but avoids unnecessary v1 complexity.</t>
-  </si>
-  <si>
-    <t>DD-005</t>
-  </si>
-  <si>
-    <t>Backup &amp; Recovery Architecture</t>
-  </si>
-  <si>
-    <t>CAP-007 Backup &amp; Recovery; CAP-003 File &amp; Data Services; CAP-004 Storage Provisioning &amp; Management; CAP-015 Compute Provisioning / Hosting; requirements for business continuity backups, backup validation and recovery testing, service recovery and recoverable operations; Availability, Reliability, Data Protection and Recoverability NFRs; CON-003 Recoverable Operations; CON-004 Proportionate Availability &amp; Resilience; CON-008 Controlled &amp; Recoverable Change; CON-013 Business Data Segregation &amp; Protection; DP-004 Design for Recoverability; DP-005 Apply Proportionate Resilience; DP-010 Prefer Controlled &amp; Reversible Change; DP-017 Protect Business Data Throughout its Lifecycle.</t>
-  </si>
-  <si>
-    <t>Business requirements fit; RPO/RTO capability; protection against accidental deletion, corruption, administrative error, workload loss, storage failure and infrastructure failure; recovery granularity; backup isolation; security; recoverability; restore testing; retention capability; operational complexity; monitoring/reporting; storage requirements; scalability; supportability; Linux/RHCSA learning alignment; integration with compute, storage and file services.</t>
-  </si>
-  <si>
-    <t>Layered backup and recovery architecture comprising short-term point-in-time recovery mechanisms, a dedicated backup service using protected backup storage, and a secondary backup copy maintained outside the primary production failure domain. Backup effectiveness will be validated through scheduled restore testing and documented recovery procedures.</t>
-  </si>
-  <si>
-    <t>A layered architecture provides protection against a broader range of failure scenarios than any single backup mechanism. Short-term point-in-time recovery provides rapid rollback for appropriate operational errors or changes, while an independent backup service and protected repository provide recoverability following data corruption, workload loss or production-storage failure. A secondary copy outside the primary failure domain provides additional protection against loss of the primary compute/storage environment. The approach supports protection at appropriate levels, including business data, system/configuration data and recoverable workload state, while allowing recovery methods and schedules to be aligned with Northwind's RPO/RTO requirements. Scheduled restore testing ensures that backup success is demonstrated through actual recoverability rather than backup-job status alone.</t>
-  </si>
-  <si>
-    <t>The layered architecture introduces additional infrastructure, storage consumption and administrative overhead compared with a simple backup approach. Snapshots or other point-in-time mechanisms remain dependent on their underlying storage and must not be treated as independent backups. A remote secondary copy does not automatically provide protection against malicious deletion or ransomware unless appropriate isolation, credentials and access controls are implemented. Backup capacity will increase according to protected data volume, backup frequency and retention requirements. Recovery procedures must be maintained and tested. Service-specific RPO/RTO values remain to be refined and may affect the eventual backup schedules, retention and recovery mechanisms selected during LLD.</t>
-  </si>
-  <si>
-    <t>1. Native/simple Linux backup architecture — scheduled file and configuration backups using Linux-native mechanisms and protected storage. 2. Dedicated backup service — central backup service/repository providing managed protection, retention and recovery of supported workloads. 3. Layered backup &amp; recovery architecture — short-term point-in-time recovery mechanisms combined with a dedicated backup service using protected backup storage and a secondary copy outside the primary production failure domain.</t>
-  </si>
-  <si>
-    <t>DD-006</t>
-  </si>
-  <si>
-    <t>Monitoring &amp; Alerting Architecture</t>
-  </si>
-  <si>
-    <t>CAP-006 Infrastructure Monitoring &amp; Alerting; CAP-012 Reporting; CAP-015 Compute Provisioning / Hosting; CAP-016 Systems Administration &amp; Management; requirements for operational monitoring and alerting, capacity and performance management, reporting and visibility, service recovery and incident investigation/troubleshooting; Availability, Reliability, Performance, Supportability and Monitoring &amp; Observability NFRs; CON-006 Observable &amp; Auditable Operations; CON-012 Supportable &amp; Maintainable Design; CON-014 Capacity &amp; Performance Visibility; DP-008 Make Operations Observable &amp; Auditable; DP-013 Design for Managed Growth; DP-016 Design for Supportability.</t>
-  </si>
-  <si>
-    <r>
-      <t>1. Native/decentralised Linux monitoring</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> — administrators use native Linux tools, scripts and scheduled checks to assess individual host and service health. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2. Dedicated central monitoring platform</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> — infrastructure and service telemetry is collected centrally to provide continuous visibility, alerting, historical data and reporting. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3. Hybrid monitoring architecture</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> — centralised monitoring provides continuous visibility, alerting, historical trends and capacity reporting, while native Linux tools remain available for detailed host-level diagnosis and troubleshooting.</t>
-    </r>
-  </si>
-  <si>
-    <t>Requirements fit; infrastructure and service visibility; proactive fault detection; service-health monitoring; alerting and escalation capability; historical metric retention; capacity/performance trending; reporting capability; Linux/RHCSA learning alignment; troubleshooting capability; operational complexity; security; scalability; supportability; monitoring-platform dependencies; integration with backup, compute, storage, networking and future application services.</t>
-  </si>
-  <si>
-    <t>Hybrid monitoring architecture consisting of a centralised monitoring and alerting service providing infrastructure and service health visibility, historical capacity/performance data, configurable threshold-based alerting and operational reporting across supported systems. Native Linux diagnostic and troubleshooting tools will remain the primary mechanism for detailed host-level investigation.</t>
-  </si>
-  <si>
-    <t>A hybrid approach provides Northwind with central operational visibility while preserving direct Linux administration and troubleshooting capability. Central monitoring enables proactive detection of host, service, storage, backup, network and resource issues; maintains historical data for capacity and performance analysis; and allows alerts to be routed to IT when defined warning or critical conditions occur. Native Linux tools complement this capability by enabling administrators to investigate the underlying cause of detected conditions directly on affected systems. This approach satisfies Northwind's monitoring, reporting and capacity-management requirements without making the monitoring platform a replacement for administrator understanding of the underlying Linux systems.</t>
-  </si>
-  <si>
-    <t>A central monitoring service introduces an additional infrastructure component that must itself be secured, patched, backed up and maintained. Failure of the monitoring platform may reduce operational visibility and create a monitoring blind spot; appropriate health checks or independent operational controls should therefore be considered. Excessive or poorly configured thresholds may cause alert fatigue, while insufficient thresholds may allow significant conditions to go undetected. Collection and retention of detailed historical metrics will consume storage and compute resources. Agent versus agentless collection, metric retention periods, thresholds, alert-routing mechanisms and monitoring-platform technology remain to be determined during subsequent design activities.</t>
+    <t>CAP-001 Identity &amp; Access Management; CAP-016 Systems Administration &amp; Management;requirements for Centralised User Identity Management, User Lifecycle Management, User Provisioning Automation, Role-Based Access Control, secure data access and administrative access; Security, Maintainability and Operational Consistency NFRs; CON-002 Least-Privilege Access; CON-005 Operational Consistency &amp; Standardisation; CON-012 Supportable &amp; Maintainable Design; DP-002 Prefer Simplicity; DP-003 Standardise Where Practical; DP-006 Enforce Least Privilege; DP-009 Treat Administrative Access as a Controlled Service; DP-015 Prefer Automation for Repeatable Operations, Not Understanding Replacement.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -721,6 +1550,21 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -746,7 +1590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -763,7 +1607,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1102,7 +1945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7EDC8A7-8218-44FF-8632-A3017F096196}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultColWidth="61.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -1144,13 +1987,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="105" x14ac:dyDescent="0.25">
@@ -1164,63 +2007,63 @@
         <v>34</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="K2" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D3" t="s">
+      <c r="G3" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H3" t="s">
-        <v>51</v>
-      </c>
-      <c r="I3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K3" t="s">
-        <v>53</v>
+      <c r="I3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="150" x14ac:dyDescent="0.25">
@@ -1228,127 +2071,318 @@
         <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="195" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="165" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="I6" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="165" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="I7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="210" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>40</v>
+      <c r="I8" s="2"/>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" ht="300" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="345" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="360" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="375" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="330" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1357,170 +2391,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C64EBDD-B34E-4461-A45B-301127E80C13}">
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:14" ht="75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="165" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F55DFBF-7C38-4C62-A958-ADC13C3CE962}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="58.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>